<commit_message>
Update metadata Excel with live public links for Word doc and Learning Designer
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Metadata_Scenario.xlsx
+++ b/Metadata_Scenario.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="d:\courses2025_2026\teaching_AI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3419F091-CC31-4C05-9B91-E2DEBBE9A882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAA625EE-2C77-4A10-9041-A522915570C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2508" yWindow="2508" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -214,12 +214,6 @@
     <t>Internet connection required (Wi-Fi recommended). One device per student or group. Free accounts for Genially, Quizizz, Canva (Canva for Education recommended). Google Sheets shared workbook pre-prepared by instructor. Basic digital skills required. No coding needed. All tools have usable free tier.</t>
   </si>
   <si>
-    <t>To be added after publishing the module on learningdesigner.org</t>
-  </si>
-  <si>
-    <t>To be added after uploading PMO_AI_Module_Pack.docx to Google Drive or OneDrive</t>
-  </si>
-  <si>
     <t>Aoude_UniversiteLibanaise_KassisCarine</t>
   </si>
   <si>
@@ -302,6 +296,12 @@
   </si>
   <si>
     <t>Lebanese University - Universite Libanaise</t>
+  </si>
+  <si>
+    <t>https://maoude.github.io/teaching-ai-pmo/PMO_AI_Module_Pack.docx</t>
+  </si>
+  <si>
+    <t>https://maoude.github.io/teaching-ai-pmo/learning_designer_pack.html</t>
   </si>
 </sst>
 </file>
@@ -468,10 +468,13 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -488,9 +491,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -733,20 +733,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:41" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="25"/>
       <c r="C1" s="25"/>
       <c r="D1" s="25"/>
       <c r="E1" s="25"/>
-      <c r="F1" s="27" t="s">
+      <c r="F1" s="28" t="s">
         <v>1</v>
       </c>
       <c r="G1" s="25"/>
       <c r="H1" s="25"/>
       <c r="I1" s="25"/>
-      <c r="J1" s="31" t="s">
+      <c r="J1" s="32" t="s">
         <v>2</v>
       </c>
       <c r="K1" s="25"/>
@@ -757,20 +757,20 @@
       <c r="P1" s="25"/>
       <c r="Q1" s="25"/>
       <c r="R1" s="25"/>
-      <c r="S1" s="28" t="s">
+      <c r="S1" s="29" t="s">
         <v>3</v>
       </c>
       <c r="T1" s="25"/>
       <c r="U1" s="25"/>
       <c r="V1" s="25"/>
       <c r="W1" s="25"/>
-      <c r="X1" s="29" t="s">
+      <c r="X1" s="30" t="s">
         <v>4</v>
       </c>
       <c r="Y1" s="25"/>
       <c r="Z1" s="25"/>
       <c r="AA1" s="25"/>
-      <c r="AB1" s="30" t="s">
+      <c r="AB1" s="31" t="s">
         <v>5</v>
       </c>
       <c r="AC1" s="25"/>
@@ -778,14 +778,14 @@
       <c r="AE1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="AF1" s="24" t="s">
+      <c r="AF1" s="26" t="s">
         <v>7</v>
       </c>
       <c r="AG1" s="25"/>
       <c r="AH1" s="25"/>
       <c r="AI1" s="25"/>
       <c r="AJ1" s="25"/>
-      <c r="AK1" s="26" t="s">
+      <c r="AK1" s="27" t="s">
         <v>8</v>
       </c>
       <c r="AL1" s="25"/>
@@ -918,94 +918,94 @@
     </row>
     <row r="3" spans="1:41" ht="202.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="G3" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="I3" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="N3" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="O3" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="P3" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q3" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="R3" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="S3" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="T3" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="U3" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="V3" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="W3" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="X3" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="Y3" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="Z3" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="AA3" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="AB3" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="AC3" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="AD3" s="3" t="s">
         <v>88</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="F3" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="H3" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="I3" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="K3" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="L3" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="M3" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="N3" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="O3" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="P3" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="Q3" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="R3" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="S3" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="T3" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="U3" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="V3" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="W3" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="X3" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="Y3" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="Z3" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="AA3" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="AB3" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="AC3" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="AD3" s="3" t="s">
-        <v>59</v>
       </c>
       <c r="AE3" s="1" t="s">
         <v>58</v>

</xml_diff>